<commit_message>
feat(facturare): update Anexa template with Cant, Invoice No., Kurs columns
New columns: D=Cant (green), K=Invoice No. (yellow), L=Kurs (yellow).
Includes storno example row (qty=-1). Yellow = optional override fields.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/jarvis/accounting/facturare/assets/Anexa_Invoice_Template.xlsx
+++ b/jarvis/accounting/facturare/assets/Anexa_Invoice_Template.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="4">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,8 +37,19 @@
     <font>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill/>
     </fill>
@@ -55,6 +66,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FFFF00"/>
         <bgColor rgb="00FFFF00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="0092D050"/>
+        <bgColor rgb="0092D050"/>
       </patternFill>
     </fill>
   </fills>
@@ -76,7 +93,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -86,6 +103,16 @@
     <xf numFmtId="4" fontId="3" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="3" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -451,18 +478,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:L4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="20" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="24" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -473,49 +503,64 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Nr. Comanda</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Model</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Culoare</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>Cant</t>
+        </is>
+      </c>
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>List Price</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>Selling Price</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>Discount</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="H2" s="7" t="inlineStr">
         <is>
           <t>Advance</t>
         </is>
       </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="I2" s="7" t="inlineStr">
         <is>
           <t>Rest</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr">
+      <c r="J2" s="7" t="inlineStr">
         <is>
           <t>VIN</t>
+        </is>
+      </c>
+      <c r="K2" s="9" t="inlineStr">
+        <is>
+          <t>Invoice No.</t>
+        </is>
+      </c>
+      <c r="L2" s="9" t="inlineStr">
+        <is>
+          <t>Kurs (EUR/RON)</t>
         </is>
       </c>
     </row>
@@ -534,21 +579,26 @@
         </is>
       </c>
       <c r="D3" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E3" s="4" t="n">
         <v>25000</v>
       </c>
-      <c r="E3" s="4" t="n">
+      <c r="F3" s="4" t="n">
         <v>24500</v>
       </c>
-      <c r="F3" s="4" t="n">
+      <c r="G3" s="4" t="n">
         <v>500</v>
       </c>
-      <c r="G3" s="4" t="n">
+      <c r="H3" s="4" t="n">
         <v>5000</v>
       </c>
-      <c r="H3" s="4" t="n">
+      <c r="I3" s="3" t="n">
         <v>19500</v>
       </c>
-      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="10" t="n"/>
+      <c r="K3" s="10" t="n"/>
+      <c r="L3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
@@ -556,30 +606,39 @@
       </c>
       <c r="B4" s="5" t="inlineStr">
         <is>
-          <t>T-Cross Style</t>
+          <t>Golf 8 Life</t>
         </is>
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>Negru</t>
+          <t>Alb</t>
         </is>
       </c>
       <c r="D4" s="6" t="n">
-        <v>22000</v>
+        <v>-1</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>21800</v>
+        <v>25000</v>
       </c>
       <c r="F4" s="6" t="n">
-        <v>200</v>
+        <v>24500</v>
       </c>
       <c r="G4" s="6" t="n">
-        <v>4000</v>
+        <v>500</v>
       </c>
       <c r="H4" s="6" t="n">
-        <v>17800</v>
-      </c>
-      <c r="I4" s="5" t="n"/>
+        <v>5000</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>19500</v>
+      </c>
+      <c r="J4" s="10" t="n"/>
+      <c r="K4" s="10" t="n">
+        <v>1</v>
+      </c>
+      <c r="L4" s="10" t="n">
+        <v>2</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
feat(facturare): add storno description column M to Anexa template
New column M (STORNO ADVANCE INVOICE) appears as first description line
on storno invoices. Only used when qty is negative and the cell is filled.
Normal invoices ignore it.

Co-Authored-By: Claude Opus 4.6 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/jarvis/accounting/facturare/assets/Anexa_Invoice_Template.xlsx
+++ b/jarvis/accounting/facturare/assets/Anexa_Invoice_Template.xlsx
@@ -478,7 +478,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -493,6 +493,7 @@
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="28" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -563,6 +564,11 @@
           <t>Kurs (EUR/RON)</t>
         </is>
       </c>
+      <c r="M2" s="9" t="inlineStr">
+        <is>
+          <t>STORNO ADVANCE INVOICE</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="n">
@@ -599,6 +605,7 @@
       <c r="J3" s="10" t="n"/>
       <c r="K3" s="10" t="n"/>
       <c r="L3" s="10" t="n"/>
+      <c r="M3" s="10" t="n"/>
     </row>
     <row r="4">
       <c r="A4" s="5" t="n">
@@ -638,6 +645,11 @@
       </c>
       <c r="L4" s="10" t="n">
         <v>2</v>
+      </c>
+      <c r="M4" s="10" t="inlineStr">
+        <is>
+          <t>9100183 / 17.04.2026</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>